<commit_message>
Initial commit of project to new branch
</commit_message>
<xml_diff>
--- a/backend/income_details.xlsx
+++ b/backend/income_details.xlsx
@@ -64,9 +64,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,120 +409,41 @@
       <c r="C1" t="str">
         <v>Date</v>
       </c>
+      <c r="D1" t="str">
+        <v>CreatedAt</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>freelance</v>
+        <v>Salary</v>
       </c>
       <c r="B2">
-        <v>100</v>
-      </c>
-      <c r="C2" s="1">
-        <v>45797.12527777778</v>
+        <v>1000</v>
+      </c>
+      <c r="C2" t="str">
+        <v>7/11/2025</v>
+      </c>
+      <c r="D2" t="str">
+        <v>7/11/2025, 9:06:29 PM</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Salary</v>
+        <v>Gift</v>
       </c>
       <c r="B3">
-        <v>1000</v>
-      </c>
-      <c r="C3" s="1">
-        <v>45789.12527777778</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>freelance</v>
-      </c>
-      <c r="B4">
-        <v>1000</v>
-      </c>
-      <c r="C4" s="1">
-        <v>45787.12527777778</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Gift</v>
-      </c>
-      <c r="B5">
-        <v>100</v>
-      </c>
-      <c r="C5" s="1">
-        <v>45787.12527777778</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Salary</v>
-      </c>
-      <c r="B6">
-        <v>2000</v>
-      </c>
-      <c r="C6" s="1">
-        <v>45759.12527777778</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>freelance</v>
-      </c>
-      <c r="B7">
-        <v>100</v>
-      </c>
-      <c r="C7" s="1">
-        <v>45759.12527777778</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Salary</v>
-      </c>
-      <c r="B8">
-        <v>1000</v>
-      </c>
-      <c r="C8" s="1">
-        <v>45748.12527777778</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Salary</v>
-      </c>
-      <c r="B9">
-        <v>1000</v>
-      </c>
-      <c r="C9" s="1">
-        <v>45717.08361111111</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>freelance</v>
-      </c>
-      <c r="B10">
-        <v>1000</v>
-      </c>
-      <c r="C10" s="1">
-        <v>45717.08361111111</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>gift</v>
-      </c>
-      <c r="B11">
-        <v>3000</v>
-      </c>
-      <c r="C11" s="1">
-        <v>45689.08361111111</v>
+        <v>300</v>
+      </c>
+      <c r="C3" t="str">
+        <v>7/9/2025</v>
+      </c>
+      <c r="D3" t="str">
+        <v>7/11/2025, 9:06:43 PM</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>